<commit_message>
update docs Sprint Backlog and UsermanualPDF for chayasak_0095
</commit_message>
<xml_diff>
--- a/Doce/Sprint Backlog.xlsx
+++ b/Doce/Sprint Backlog.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="56">
   <si>
     <t>Sprint No.</t>
   </si>
@@ -55,10 +55,16 @@
     <t>As a user, I want my account and information to be removed from the system when I am no longer want to be apart of this community.</t>
   </si>
   <si>
+    <t>Doc</t>
+  </si>
+  <si>
     <t>A-Dapt Blueprint</t>
   </si>
   <si>
     <t>EveryOne</t>
+  </si>
+  <si>
+    <t>Frontend</t>
   </si>
   <si>
     <t>ออกแบบ Frontend ใน Figma เพิ่มปุ่มลบและยืนยันการลบบัญชีผู้ใช้งาน</t>
@@ -103,6 +109,9 @@
     <t>Chaysak/Phakhawat</t>
   </si>
   <si>
+    <t>Backend</t>
+  </si>
+  <si>
     <t>เชื่อม และ แก้ไข Database  สำหรับลบข้อมูล</t>
   </si>
   <si>
@@ -139,6 +148,9 @@
     <t>แก้ไขบัคที่พบ</t>
   </si>
   <si>
+    <t>Test</t>
+  </si>
+  <si>
     <t>เขียนโค้ด test UAT และทำการทดสอบ</t>
   </si>
   <si>
@@ -157,7 +169,13 @@
     <t>ทำ Report API Test</t>
   </si>
   <si>
+    <t>Depoy</t>
+  </si>
+  <si>
     <t xml:space="preserve">Deploy </t>
+  </si>
+  <si>
+    <t>Papop/Phakhawat</t>
   </si>
   <si>
     <t>ศึกษาและทดลองรันระบบบนเซิฟเวอร์จริง</t>
@@ -167,7 +185,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -181,6 +199,7 @@
     </font>
     <font/>
     <font>
+      <sz val="18.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -189,6 +208,11 @@
       <sz val="20.0"/>
       <color rgb="FF000000"/>
       <name val="&quot;Cordia New&quot;"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -317,7 +341,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -342,11 +366,16 @@
     <xf borderId="10" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="10" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="10" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="11" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -377,7 +406,8 @@
     <xf borderId="10" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="10" fillId="2" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="10" fillId="2" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -482,11 +512,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1606400463"/>
-        <c:axId val="747772552"/>
+        <c:axId val="1327943856"/>
+        <c:axId val="620746775"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1606400463"/>
+        <c:axId val="1327943856"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -538,10 +568,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="747772552"/>
+        <c:crossAx val="620746775"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="747772552"/>
+        <c:axId val="620746775"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -616,7 +646,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1606400463"/>
+        <c:crossAx val="1327943856"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -647,9 +677,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>57150</xdr:colOff>
+      <xdr:colOff>419100</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="5715000" cy="3533775"/>
     <xdr:graphicFrame>
@@ -1011,13 +1041,15 @@
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="12"/>
+      <c r="C4" s="12" t="s">
+        <v>14</v>
+      </c>
       <c r="D4" s="11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G4" s="11">
         <v>0.0</v>
@@ -1058,15 +1090,17 @@
     <row r="5">
       <c r="A5" s="14"/>
       <c r="B5" s="14"/>
-      <c r="C5" s="12"/>
+      <c r="C5" s="15" t="s">
+        <v>17</v>
+      </c>
       <c r="D5" s="11" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E5" s="11">
         <v>3.0</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G5" s="11">
         <v>3.0</v>
@@ -1090,8 +1124,8 @@
         <v>0.0</v>
       </c>
       <c r="N5" s="1"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
@@ -1107,15 +1141,15 @@
     <row r="6">
       <c r="A6" s="14"/>
       <c r="B6" s="14"/>
-      <c r="C6" s="12"/>
+      <c r="C6" s="14"/>
       <c r="D6" s="11" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E6" s="11">
         <v>3.0</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G6" s="11">
         <v>3.0</v>
@@ -1156,15 +1190,15 @@
     <row r="7">
       <c r="A7" s="14"/>
       <c r="B7" s="14"/>
-      <c r="C7" s="12"/>
+      <c r="C7" s="14"/>
       <c r="D7" s="11" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E7" s="11">
         <v>3.0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G7" s="11">
         <v>3.0</v>
@@ -1205,15 +1239,15 @@
     <row r="8">
       <c r="A8" s="14"/>
       <c r="B8" s="14"/>
-      <c r="C8" s="12"/>
+      <c r="C8" s="8"/>
       <c r="D8" s="11" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E8" s="11">
         <v>3.0</v>
       </c>
-      <c r="F8" s="16" t="s">
-        <v>23</v>
+      <c r="F8" s="17" t="s">
+        <v>25</v>
       </c>
       <c r="G8" s="11">
         <v>0.0</v>
@@ -1238,8 +1272,8 @@
       </c>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
-      <c r="P8" s="15" t="s">
-        <v>24</v>
+      <c r="P8" s="16" t="s">
+        <v>26</v>
       </c>
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
@@ -1256,15 +1290,17 @@
     <row r="9">
       <c r="A9" s="14"/>
       <c r="B9" s="14"/>
-      <c r="C9" s="12"/>
+      <c r="C9" s="15" t="s">
+        <v>14</v>
+      </c>
       <c r="D9" s="11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E9" s="11">
         <v>3.0</v>
       </c>
-      <c r="F9" s="16" t="s">
-        <v>26</v>
+      <c r="F9" s="17" t="s">
+        <v>28</v>
       </c>
       <c r="G9" s="11">
         <v>0.0</v>
@@ -1289,8 +1325,8 @@
       </c>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
-      <c r="P9" s="17" t="s">
-        <v>27</v>
+      <c r="P9" s="18" t="s">
+        <v>29</v>
       </c>
       <c r="Q9" s="6"/>
       <c r="R9" s="6"/>
@@ -1300,22 +1336,22 @@
       <c r="V9" s="6"/>
       <c r="W9" s="6"/>
       <c r="X9" s="7"/>
-      <c r="Y9" s="18"/>
-      <c r="Z9" s="18"/>
-      <c r="AA9" s="18"/>
+      <c r="Y9" s="19"/>
+      <c r="Z9" s="19"/>
+      <c r="AA9" s="19"/>
     </row>
     <row r="10">
       <c r="A10" s="14"/>
       <c r="B10" s="14"/>
-      <c r="C10" s="12"/>
+      <c r="C10" s="8"/>
       <c r="D10" s="11" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E10" s="11">
         <v>3.0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G10" s="11">
         <v>0.0</v>
@@ -1340,45 +1376,47 @@
       </c>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
-      <c r="P10" s="19"/>
-      <c r="Q10" s="19"/>
-      <c r="R10" s="20">
+      <c r="P10" s="20"/>
+      <c r="Q10" s="20"/>
+      <c r="R10" s="21">
         <v>1.0</v>
       </c>
-      <c r="S10" s="20">
+      <c r="S10" s="21">
         <v>2.0</v>
       </c>
-      <c r="T10" s="20">
+      <c r="T10" s="21">
         <v>3.0</v>
       </c>
-      <c r="U10" s="20">
+      <c r="U10" s="21">
         <v>4.0</v>
       </c>
-      <c r="V10" s="20">
+      <c r="V10" s="21">
         <v>5.0</v>
       </c>
-      <c r="W10" s="20">
+      <c r="W10" s="21">
         <v>6.0</v>
       </c>
-      <c r="X10" s="20">
+      <c r="X10" s="21">
         <v>7.0</v>
       </c>
-      <c r="Y10" s="18"/>
-      <c r="Z10" s="18"/>
-      <c r="AA10" s="18"/>
+      <c r="Y10" s="19"/>
+      <c r="Z10" s="19"/>
+      <c r="AA10" s="19"/>
     </row>
     <row r="11">
       <c r="A11" s="14"/>
       <c r="B11" s="14"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="16" t="s">
-        <v>30</v>
+      <c r="C11" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>33</v>
       </c>
       <c r="E11" s="11">
         <v>3.0</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G11" s="11">
         <v>0.0</v>
@@ -1403,56 +1441,56 @@
       </c>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
-      <c r="P11" s="21" t="s">
-        <v>31</v>
+      <c r="P11" s="22" t="s">
+        <v>34</v>
       </c>
-      <c r="Q11" s="21" t="s">
-        <v>32</v>
+      <c r="Q11" s="22" t="s">
+        <v>35</v>
       </c>
-      <c r="R11" s="20">
-        <f>SUM(G5:G27)</f>
+      <c r="R11" s="21">
+        <f>SUM(G5:G25)</f>
         <v>9</v>
       </c>
-      <c r="S11" s="20">
+      <c r="S11" s="21">
         <f t="shared" ref="S11:X11" si="1">SUM(H5:H23)</f>
         <v>12</v>
       </c>
-      <c r="T11" s="20">
+      <c r="T11" s="21">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="U11" s="20">
+      <c r="U11" s="21">
         <f t="shared" si="1"/>
         <v>21</v>
       </c>
-      <c r="V11" s="20">
+      <c r="V11" s="21">
         <f t="shared" si="1"/>
         <v>51</v>
       </c>
-      <c r="W11" s="20">
+      <c r="W11" s="21">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="X11" s="20">
+      <c r="X11" s="21">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="Y11" s="18"/>
-      <c r="Z11" s="18"/>
-      <c r="AA11" s="18"/>
+      <c r="Y11" s="19"/>
+      <c r="Z11" s="19"/>
+      <c r="AA11" s="19"/>
     </row>
     <row r="12">
       <c r="A12" s="14"/>
       <c r="B12" s="14"/>
-      <c r="C12" s="12"/>
+      <c r="C12" s="14"/>
       <c r="D12" s="11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E12" s="11">
         <v>3.0</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G12" s="11">
         <v>0.0</v>
@@ -1477,56 +1515,56 @@
       </c>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
-      <c r="P12" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q12" s="21" t="s">
+      <c r="P12" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="R12" s="20">
-        <f t="shared" ref="R12:X12" si="2">SUM($E$4:$E$27)*(1-R10/10)</f>
+      <c r="Q12" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="R12" s="21">
+        <f t="shared" ref="R12:X12" si="2">SUM($E$4:$E$25)*(1-R10/10)</f>
         <v>70.2</v>
       </c>
-      <c r="S12" s="20">
+      <c r="S12" s="21">
         <f t="shared" si="2"/>
         <v>62.4</v>
       </c>
-      <c r="T12" s="20">
+      <c r="T12" s="21">
         <f t="shared" si="2"/>
         <v>54.6</v>
       </c>
-      <c r="U12" s="20">
+      <c r="U12" s="21">
         <f t="shared" si="2"/>
         <v>46.8</v>
       </c>
-      <c r="V12" s="20">
+      <c r="V12" s="21">
         <f t="shared" si="2"/>
         <v>39</v>
       </c>
-      <c r="W12" s="20">
+      <c r="W12" s="21">
         <f t="shared" si="2"/>
         <v>31.2</v>
       </c>
-      <c r="X12" s="20">
+      <c r="X12" s="21">
         <f t="shared" si="2"/>
         <v>23.4</v>
       </c>
-      <c r="Y12" s="18"/>
-      <c r="Z12" s="18"/>
-      <c r="AA12" s="18"/>
+      <c r="Y12" s="19"/>
+      <c r="Z12" s="19"/>
+      <c r="AA12" s="19"/>
     </row>
     <row r="13">
       <c r="A13" s="14"/>
       <c r="B13" s="14"/>
-      <c r="C13" s="12"/>
+      <c r="C13" s="14"/>
       <c r="D13" s="11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E13" s="11">
         <v>3.0</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G13" s="11">
         <v>0.0</v>
@@ -1567,15 +1605,15 @@
     <row r="14">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
-      <c r="C14" s="12"/>
+      <c r="C14" s="14"/>
       <c r="D14" s="11" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E14" s="11">
         <v>6.0</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G14" s="11">
         <v>0.0</v>
@@ -1616,15 +1654,15 @@
     <row r="15">
       <c r="A15" s="14"/>
       <c r="B15" s="14"/>
-      <c r="C15" s="12"/>
+      <c r="C15" s="14"/>
       <c r="D15" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E15" s="11">
         <v>6.0</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G15" s="11">
         <v>0.0</v>
@@ -1665,15 +1703,15 @@
     <row r="16">
       <c r="A16" s="14"/>
       <c r="B16" s="14"/>
-      <c r="C16" s="12"/>
+      <c r="C16" s="14"/>
       <c r="D16" s="11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E16" s="11">
         <v>6.0</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G16" s="11">
         <v>0.0</v>
@@ -1714,15 +1752,15 @@
     <row r="17">
       <c r="A17" s="14"/>
       <c r="B17" s="14"/>
-      <c r="C17" s="12"/>
+      <c r="C17" s="14"/>
       <c r="D17" s="11" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E17" s="11">
         <v>6.0</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G17" s="11">
         <v>0.0</v>
@@ -1763,15 +1801,15 @@
     <row r="18">
       <c r="A18" s="14"/>
       <c r="B18" s="14"/>
-      <c r="C18" s="12"/>
+      <c r="C18" s="14"/>
       <c r="D18" s="11" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E18" s="11">
         <v>6.0</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G18" s="11">
         <v>0.0</v>
@@ -1812,15 +1850,15 @@
     <row r="19">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
-      <c r="C19" s="12"/>
+      <c r="C19" s="8"/>
       <c r="D19" s="11" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E19" s="11">
         <v>9.0</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G19" s="11">
         <v>0.0</v>
@@ -1861,15 +1899,17 @@
     <row r="20">
       <c r="A20" s="14"/>
       <c r="B20" s="14"/>
-      <c r="C20" s="12"/>
+      <c r="C20" s="15" t="s">
+        <v>45</v>
+      </c>
       <c r="D20" s="11" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E20" s="11">
         <v>3.0</v>
       </c>
-      <c r="F20" s="16" t="s">
-        <v>43</v>
+      <c r="F20" s="17" t="s">
+        <v>47</v>
       </c>
       <c r="G20" s="11">
         <v>0.0</v>
@@ -1910,15 +1950,15 @@
     <row r="21">
       <c r="A21" s="14"/>
       <c r="B21" s="14"/>
-      <c r="C21" s="12"/>
+      <c r="C21" s="14"/>
       <c r="D21" s="11" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E21" s="11">
         <v>3.0</v>
       </c>
-      <c r="F21" s="16" t="s">
-        <v>45</v>
+      <c r="F21" s="17" t="s">
+        <v>49</v>
       </c>
       <c r="G21" s="11">
         <v>0.0</v>
@@ -1929,7 +1969,7 @@
       <c r="I21" s="11">
         <v>0.0</v>
       </c>
-      <c r="J21" s="22">
+      <c r="J21" s="23">
         <v>0.0</v>
       </c>
       <c r="K21" s="11">
@@ -1959,15 +1999,15 @@
     <row r="22">
       <c r="A22" s="14"/>
       <c r="B22" s="14"/>
-      <c r="C22" s="12"/>
+      <c r="C22" s="14"/>
       <c r="D22" s="11" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E22" s="11">
         <v>3.0</v>
       </c>
-      <c r="F22" s="16" t="s">
-        <v>43</v>
+      <c r="F22" s="17" t="s">
+        <v>47</v>
       </c>
       <c r="G22" s="11">
         <v>0.0</v>
@@ -2008,15 +2048,15 @@
     <row r="23">
       <c r="A23" s="14"/>
       <c r="B23" s="14"/>
-      <c r="C23" s="12"/>
+      <c r="C23" s="8"/>
       <c r="D23" s="11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E23" s="11">
         <v>3.0</v>
       </c>
-      <c r="F23" s="16" t="s">
-        <v>45</v>
+      <c r="F23" s="17" t="s">
+        <v>49</v>
       </c>
       <c r="G23" s="11">
         <v>0.0</v>
@@ -2057,17 +2097,23 @@
     <row r="24">
       <c r="A24" s="14"/>
       <c r="B24" s="14"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
-      <c r="J24" s="13"/>
-      <c r="K24" s="13"/>
-      <c r="L24" s="13"/>
-      <c r="M24" s="13"/>
+      <c r="C24" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="E24" s="25"/>
+      <c r="F24" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="G24" s="26"/>
+      <c r="H24" s="25"/>
+      <c r="I24" s="25"/>
+      <c r="J24" s="25"/>
+      <c r="K24" s="25"/>
+      <c r="L24" s="25"/>
+      <c r="M24" s="25"/>
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
       <c r="P24" s="1"/>
@@ -2086,17 +2132,21 @@
     <row r="25">
       <c r="A25" s="14"/>
       <c r="B25" s="14"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="13"/>
-      <c r="I25" s="13"/>
-      <c r="J25" s="13"/>
-      <c r="K25" s="13"/>
-      <c r="L25" s="13"/>
-      <c r="M25" s="13"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="E25" s="25"/>
+      <c r="F25" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="G25" s="25"/>
+      <c r="H25" s="25"/>
+      <c r="I25" s="25"/>
+      <c r="J25" s="25"/>
+      <c r="K25" s="25"/>
+      <c r="L25" s="25"/>
+      <c r="M25" s="25"/>
       <c r="N25" s="1"/>
       <c r="O25" s="1"/>
       <c r="P25" s="1"/>
@@ -2115,19 +2165,17 @@
     <row r="26">
       <c r="A26" s="14"/>
       <c r="B26" s="14"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="E26" s="24"/>
-      <c r="F26" s="23"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="24"/>
-      <c r="I26" s="24"/>
-      <c r="J26" s="24"/>
-      <c r="K26" s="24"/>
-      <c r="L26" s="24"/>
-      <c r="M26" s="24"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="27"/>
+      <c r="I26" s="27"/>
+      <c r="J26" s="27"/>
+      <c r="K26" s="27"/>
+      <c r="L26" s="27"/>
+      <c r="M26" s="27"/>
       <c r="N26" s="1"/>
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
@@ -2146,19 +2194,17 @@
     <row r="27">
       <c r="A27" s="8"/>
       <c r="B27" s="8"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="13"/>
-      <c r="J27" s="13"/>
-      <c r="K27" s="13"/>
-      <c r="L27" s="13"/>
-      <c r="M27" s="13"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="27"/>
+      <c r="J27" s="27"/>
+      <c r="K27" s="27"/>
+      <c r="L27" s="27"/>
+      <c r="M27" s="27"/>
       <c r="N27" s="1"/>
       <c r="O27" s="1"/>
       <c r="P27" s="1"/>
@@ -30595,7 +30641,13 @@
       <c r="AA1007" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="14">
+    <mergeCell ref="G2:M2"/>
+    <mergeCell ref="P9:X9"/>
+    <mergeCell ref="C5:C8"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="C20:C23"/>
+    <mergeCell ref="C24:C25"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:D3"/>
@@ -30603,8 +30655,7 @@
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="A4:A27"/>
     <mergeCell ref="B4:B27"/>
-    <mergeCell ref="G2:M2"/>
-    <mergeCell ref="P9:X9"/>
+    <mergeCell ref="C11:C19"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>